<commit_message>
Se puso en formato fecha
</commit_message>
<xml_diff>
--- a/date_wanted.xlsx
+++ b/date_wanted.xlsx
@@ -463,12 +463,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sergio Domingo</t>
+          <t>Gonzalo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Larrea</t>
+          <t>Alarcon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -478,12 +478,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>24 ene 1959</t>
+          <t>03/04/1997</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14.079.784</t>
+          <t>40.243.112</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>